<commit_message>
Redesign for multi-trait analysis — all traits processed in one run
sample_data.xlsx: wide-format template with 5 sample traits (GrainYield,
PlantHeight, SPAD, SeedWeight, Biomass); pairs named TraitName_Yp / TraitName_Ys.

stress_tolerance_indices.R: auto-detects all trait pairs from column names,
loops through every trait, outputs per-trait biplots + lollipops, a faceted
bar chart across all traits, a cross-trait STI heatmap, a combined CSV, and
a multi-sheet Excel results workbook.

build_sample_excel.py: updated to generate the new multi-trait layout.

https://claude.ai/code/session_01QoruzK8a1BEVMKvZxSHE2H
</commit_message>
<xml_diff>
--- a/sample_data.xlsx
+++ b/sample_data.xlsx
@@ -53,7 +53,7 @@
       <sz val="13"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -72,7 +72,27 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="005a8a5e"/>
+        <fgColor rgb="001a3a5e"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="005e1a1a"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="005e4a1a"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="003a1a5e"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00f5f5f5"/>
       </patternFill>
     </fill>
     <fill>
@@ -82,7 +102,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00f5f5f5"/>
+        <fgColor rgb="005a8a5e"/>
       </patternFill>
     </fill>
   </fills>
@@ -104,7 +124,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -112,40 +132,68 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -516,269 +564,640 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D23"/>
+  <dimension ref="A1:K24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Plant Stress Tolerance Indices — Input Data</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="32" customHeight="1">
+          <t>Plant Stress Tolerance Indices — Multi-Trait Input Data</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="30" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Fill in Yp (non-stress) and Ys (stress) yield values for each genotype. Trait can be grain yield, biomass, or any stress-sensitive variable.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="40" customHeight="1">
-      <c r="A3" s="3" t="inlineStr">
+          <t>Add or rename trait columns following the pattern  TraitName_Yp  /  TraitName_Ys. Yp = non-stress value, Ys = stress value. The R script detects all pairs automatically.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="3" t="inlineStr"/>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>GrainYield</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>PlantHeight</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>SPAD</t>
+        </is>
+      </c>
+      <c r="H3" s="7" t="inlineStr">
+        <is>
+          <t>SeedWeight</t>
+        </is>
+      </c>
+      <c r="J3" s="8" t="inlineStr">
+        <is>
+          <t>Biomass</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="38" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>Genotype</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>Yp
-(Non-Stress Yield)</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>Ys
-(Stress Yield)</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>Notes (optional)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>GrainYield_Yp
+(Non-Stress)</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="inlineStr">
+        <is>
+          <t>GrainYield_Ys
+(Stress)</t>
+        </is>
+      </c>
+      <c r="D4" s="10" t="inlineStr">
+        <is>
+          <t>PlantHeight_Yp
+(Non-Stress)</t>
+        </is>
+      </c>
+      <c r="E4" s="10" t="inlineStr">
+        <is>
+          <t>PlantHeight_Ys
+(Stress)</t>
+        </is>
+      </c>
+      <c r="F4" s="11" t="inlineStr">
+        <is>
+          <t>SPAD_Yp
+(Non-Stress)</t>
+        </is>
+      </c>
+      <c r="G4" s="11" t="inlineStr">
+        <is>
+          <t>SPAD_Ys
+(Stress)</t>
+        </is>
+      </c>
+      <c r="H4" s="12" t="inlineStr">
+        <is>
+          <t>SeedWeight_Yp
+(Non-Stress)</t>
+        </is>
+      </c>
+      <c r="I4" s="12" t="inlineStr">
+        <is>
+          <t>SeedWeight_Ys
+(Stress)</t>
+        </is>
+      </c>
+      <c r="J4" s="13" t="inlineStr">
+        <is>
+          <t>Biomass_Yp
+(Non-Stress)</t>
+        </is>
+      </c>
+      <c r="K4" s="13" t="inlineStr">
+        <is>
+          <t>Biomass_Ys
+(Stress)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="A5" s="14" t="inlineStr">
         <is>
           <t>G1</t>
         </is>
       </c>
-      <c r="B4" s="5" t="n">
+      <c r="B5" s="15" t="n">
         <v>4.2</v>
       </c>
-      <c r="C4" s="5" t="n">
+      <c r="C5" s="15" t="n">
         <v>2.8</v>
       </c>
-      <c r="D4" s="4" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="6" t="inlineStr">
+      <c r="D5" s="15" t="n">
+        <v>92</v>
+      </c>
+      <c r="E5" s="15" t="n">
+        <v>78</v>
+      </c>
+      <c r="F5" s="15" t="n">
+        <v>44.2</v>
+      </c>
+      <c r="G5" s="15" t="n">
+        <v>36.1</v>
+      </c>
+      <c r="H5" s="15" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="I5" s="15" t="n">
+        <v>14.2</v>
+      </c>
+      <c r="J5" s="15" t="n">
+        <v>8.1</v>
+      </c>
+      <c r="K5" s="15" t="n">
+        <v>5.8</v>
+      </c>
+    </row>
+    <row r="6" ht="18" customHeight="1">
+      <c r="A6" s="16" t="inlineStr">
         <is>
           <t>G2</t>
         </is>
       </c>
-      <c r="B5" s="7" t="n">
+      <c r="B6" s="17" t="n">
         <v>3.85</v>
       </c>
-      <c r="C5" s="7" t="n">
+      <c r="C6" s="17" t="n">
         <v>2.6</v>
       </c>
-      <c r="D5" s="6" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="D6" s="17" t="n">
+        <v>88</v>
+      </c>
+      <c r="E6" s="17" t="n">
+        <v>74</v>
+      </c>
+      <c r="F6" s="17" t="n">
+        <v>42.8</v>
+      </c>
+      <c r="G6" s="17" t="n">
+        <v>33.5</v>
+      </c>
+      <c r="H6" s="17" t="n">
+        <v>17.2</v>
+      </c>
+      <c r="I6" s="17" t="n">
+        <v>12.8</v>
+      </c>
+      <c r="J6" s="17" t="n">
+        <v>7.6</v>
+      </c>
+      <c r="K6" s="17" t="n">
+        <v>5.2</v>
+      </c>
+    </row>
+    <row r="7" ht="18" customHeight="1">
+      <c r="A7" s="14" t="inlineStr">
         <is>
           <t>G3</t>
         </is>
       </c>
-      <c r="B6" s="5" t="n">
+      <c r="B7" s="15" t="n">
         <v>4.6</v>
       </c>
-      <c r="C6" s="5" t="n">
+      <c r="C7" s="15" t="n">
         <v>2.5</v>
       </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>drought tolerant check</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="6" t="inlineStr">
+      <c r="D7" s="15" t="n">
+        <v>95</v>
+      </c>
+      <c r="E7" s="15" t="n">
+        <v>80</v>
+      </c>
+      <c r="F7" s="15" t="n">
+        <v>45.6</v>
+      </c>
+      <c r="G7" s="15" t="n">
+        <v>34.8</v>
+      </c>
+      <c r="H7" s="15" t="n">
+        <v>19</v>
+      </c>
+      <c r="I7" s="15" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="J7" s="15" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="K7" s="15" t="n">
+        <v>5.5</v>
+      </c>
+    </row>
+    <row r="8" ht="18" customHeight="1">
+      <c r="A8" s="16" t="inlineStr">
         <is>
           <t>G4</t>
         </is>
       </c>
-      <c r="B7" s="7" t="n">
+      <c r="B8" s="17" t="n">
         <v>3.5</v>
       </c>
-      <c r="C7" s="7" t="n">
+      <c r="C8" s="17" t="n">
         <v>2.4</v>
       </c>
-      <c r="D7" s="6" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="D8" s="17" t="n">
+        <v>84</v>
+      </c>
+      <c r="E8" s="17" t="n">
+        <v>70</v>
+      </c>
+      <c r="F8" s="17" t="n">
+        <v>40.1</v>
+      </c>
+      <c r="G8" s="17" t="n">
+        <v>32</v>
+      </c>
+      <c r="H8" s="17" t="n">
+        <v>16.5</v>
+      </c>
+      <c r="I8" s="17" t="n">
+        <v>12.1</v>
+      </c>
+      <c r="J8" s="17" t="n">
+        <v>7</v>
+      </c>
+      <c r="K8" s="17" t="n">
+        <v>4.9</v>
+      </c>
+    </row>
+    <row r="9" ht="18" customHeight="1">
+      <c r="A9" s="14" t="inlineStr">
         <is>
           <t>G5</t>
         </is>
       </c>
-      <c r="B8" s="5" t="n">
+      <c r="B9" s="15" t="n">
         <v>4.1</v>
       </c>
-      <c r="C8" s="5" t="n">
+      <c r="C9" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="D8" s="4" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="6" t="inlineStr">
+      <c r="D9" s="15" t="n">
+        <v>90</v>
+      </c>
+      <c r="E9" s="15" t="n">
+        <v>79</v>
+      </c>
+      <c r="F9" s="15" t="n">
+        <v>43.5</v>
+      </c>
+      <c r="G9" s="15" t="n">
+        <v>37.2</v>
+      </c>
+      <c r="H9" s="15" t="n">
+        <v>18</v>
+      </c>
+      <c r="I9" s="15" t="n">
+        <v>14.8</v>
+      </c>
+      <c r="J9" s="15" t="n">
+        <v>7.9</v>
+      </c>
+      <c r="K9" s="15" t="n">
+        <v>6.1</v>
+      </c>
+    </row>
+    <row r="10" ht="18" customHeight="1">
+      <c r="A10" s="16" t="inlineStr">
         <is>
           <t>G6</t>
         </is>
       </c>
-      <c r="B9" s="7" t="n">
+      <c r="B10" s="17" t="n">
         <v>5</v>
       </c>
-      <c r="C9" s="7" t="n">
+      <c r="C10" s="17" t="n">
         <v>2.7</v>
       </c>
-      <c r="D9" s="6" t="inlineStr">
-        <is>
-          <t>high yielding check</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
+      <c r="D10" s="17" t="n">
+        <v>98</v>
+      </c>
+      <c r="E10" s="17" t="n">
+        <v>82</v>
+      </c>
+      <c r="F10" s="17" t="n">
+        <v>47</v>
+      </c>
+      <c r="G10" s="17" t="n">
+        <v>35.5</v>
+      </c>
+      <c r="H10" s="17" t="n">
+        <v>20.1</v>
+      </c>
+      <c r="I10" s="17" t="n">
+        <v>13.9</v>
+      </c>
+      <c r="J10" s="17" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="K10" s="17" t="n">
+        <v>5.6</v>
+      </c>
+    </row>
+    <row r="11" ht="18" customHeight="1">
+      <c r="A11" s="14" t="inlineStr">
         <is>
           <t>G7</t>
         </is>
       </c>
-      <c r="B10" s="5" t="n">
+      <c r="B11" s="15" t="n">
         <v>3.7</v>
       </c>
-      <c r="C10" s="5" t="n">
+      <c r="C11" s="15" t="n">
         <v>2.2</v>
       </c>
-      <c r="D10" s="4" t="inlineStr">
-        <is>
-          <t>sensitive check</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="6" t="inlineStr">
+      <c r="D11" s="15" t="n">
+        <v>86</v>
+      </c>
+      <c r="E11" s="15" t="n">
+        <v>71</v>
+      </c>
+      <c r="F11" s="15" t="n">
+        <v>41.3</v>
+      </c>
+      <c r="G11" s="15" t="n">
+        <v>31</v>
+      </c>
+      <c r="H11" s="15" t="n">
+        <v>16.8</v>
+      </c>
+      <c r="I11" s="15" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="J11" s="15" t="n">
+        <v>7.2</v>
+      </c>
+      <c r="K11" s="15" t="n">
+        <v>4.6</v>
+      </c>
+    </row>
+    <row r="12" ht="18" customHeight="1">
+      <c r="A12" s="16" t="inlineStr">
         <is>
           <t>G8</t>
         </is>
       </c>
-      <c r="B11" s="7" t="n">
+      <c r="B12" s="17" t="n">
         <v>4.8</v>
       </c>
-      <c r="C11" s="7" t="n">
+      <c r="C12" s="17" t="n">
         <v>3.1</v>
       </c>
-      <c r="D11" s="6" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
+      <c r="D12" s="17" t="n">
+        <v>96</v>
+      </c>
+      <c r="E12" s="17" t="n">
+        <v>83</v>
+      </c>
+      <c r="F12" s="17" t="n">
+        <v>46.1</v>
+      </c>
+      <c r="G12" s="17" t="n">
+        <v>38</v>
+      </c>
+      <c r="H12" s="17" t="n">
+        <v>19.5</v>
+      </c>
+      <c r="I12" s="17" t="n">
+        <v>15.2</v>
+      </c>
+      <c r="J12" s="17" t="n">
+        <v>9.1</v>
+      </c>
+      <c r="K12" s="17" t="n">
+        <v>6.3</v>
+      </c>
+    </row>
+    <row r="13" ht="18" customHeight="1">
+      <c r="A13" s="14" t="inlineStr">
         <is>
           <t>G9</t>
         </is>
       </c>
-      <c r="B12" s="5" t="n">
+      <c r="B13" s="15" t="n">
         <v>4.3</v>
       </c>
-      <c r="C12" s="5" t="n">
+      <c r="C13" s="15" t="n">
         <v>2.9</v>
       </c>
-      <c r="D12" s="4" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="6" t="inlineStr">
+      <c r="D13" s="15" t="n">
+        <v>91</v>
+      </c>
+      <c r="E13" s="15" t="n">
+        <v>80</v>
+      </c>
+      <c r="F13" s="15" t="n">
+        <v>44.8</v>
+      </c>
+      <c r="G13" s="15" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="H13" s="15" t="n">
+        <v>18.3</v>
+      </c>
+      <c r="I13" s="15" t="n">
+        <v>14.6</v>
+      </c>
+      <c r="J13" s="15" t="n">
+        <v>8.300000000000001</v>
+      </c>
+      <c r="K13" s="15" t="n">
+        <v>5.9</v>
+      </c>
+    </row>
+    <row r="14" ht="18" customHeight="1">
+      <c r="A14" s="16" t="inlineStr">
         <is>
           <t>G10</t>
         </is>
       </c>
-      <c r="B13" s="7" t="n">
+      <c r="B14" s="17" t="n">
         <v>3.95</v>
       </c>
-      <c r="C13" s="7" t="n">
+      <c r="C14" s="17" t="n">
         <v>2.5</v>
       </c>
-      <c r="D13" s="6" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="4" t="n"/>
-      <c r="B14" s="8" t="n"/>
-      <c r="C14" s="8" t="n"/>
-      <c r="D14" s="4" t="n"/>
+      <c r="D14" s="17" t="n">
+        <v>89</v>
+      </c>
+      <c r="E14" s="17" t="n">
+        <v>75</v>
+      </c>
+      <c r="F14" s="17" t="n">
+        <v>43</v>
+      </c>
+      <c r="G14" s="17" t="n">
+        <v>33.8</v>
+      </c>
+      <c r="H14" s="17" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="I14" s="17" t="n">
+        <v>12.6</v>
+      </c>
+      <c r="J14" s="17" t="n">
+        <v>7.75</v>
+      </c>
+      <c r="K14" s="17" t="n">
+        <v>5.1</v>
+      </c>
     </row>
     <row r="15">
-      <c r="A15" s="6" t="n"/>
-      <c r="B15" s="9" t="n"/>
-      <c r="C15" s="9" t="n"/>
-      <c r="D15" s="6" t="n"/>
+      <c r="A15" s="14" t="n"/>
+      <c r="B15" s="18" t="n"/>
+      <c r="C15" s="18" t="n"/>
+      <c r="D15" s="18" t="n"/>
+      <c r="E15" s="18" t="n"/>
+      <c r="F15" s="18" t="n"/>
+      <c r="G15" s="18" t="n"/>
+      <c r="H15" s="18" t="n"/>
+      <c r="I15" s="18" t="n"/>
+      <c r="J15" s="18" t="n"/>
+      <c r="K15" s="18" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="4" t="n"/>
-      <c r="B16" s="8" t="n"/>
-      <c r="C16" s="8" t="n"/>
-      <c r="D16" s="4" t="n"/>
+      <c r="A16" s="16" t="n"/>
+      <c r="B16" s="19" t="n"/>
+      <c r="C16" s="19" t="n"/>
+      <c r="D16" s="19" t="n"/>
+      <c r="E16" s="19" t="n"/>
+      <c r="F16" s="19" t="n"/>
+      <c r="G16" s="19" t="n"/>
+      <c r="H16" s="19" t="n"/>
+      <c r="I16" s="19" t="n"/>
+      <c r="J16" s="19" t="n"/>
+      <c r="K16" s="19" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="6" t="n"/>
-      <c r="B17" s="9" t="n"/>
-      <c r="C17" s="9" t="n"/>
-      <c r="D17" s="6" t="n"/>
+      <c r="A17" s="14" t="n"/>
+      <c r="B17" s="18" t="n"/>
+      <c r="C17" s="18" t="n"/>
+      <c r="D17" s="18" t="n"/>
+      <c r="E17" s="18" t="n"/>
+      <c r="F17" s="18" t="n"/>
+      <c r="G17" s="18" t="n"/>
+      <c r="H17" s="18" t="n"/>
+      <c r="I17" s="18" t="n"/>
+      <c r="J17" s="18" t="n"/>
+      <c r="K17" s="18" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="4" t="n"/>
-      <c r="B18" s="8" t="n"/>
-      <c r="C18" s="8" t="n"/>
-      <c r="D18" s="4" t="n"/>
+      <c r="A18" s="16" t="n"/>
+      <c r="B18" s="19" t="n"/>
+      <c r="C18" s="19" t="n"/>
+      <c r="D18" s="19" t="n"/>
+      <c r="E18" s="19" t="n"/>
+      <c r="F18" s="19" t="n"/>
+      <c r="G18" s="19" t="n"/>
+      <c r="H18" s="19" t="n"/>
+      <c r="I18" s="19" t="n"/>
+      <c r="J18" s="19" t="n"/>
+      <c r="K18" s="19" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="6" t="n"/>
-      <c r="B19" s="9" t="n"/>
-      <c r="C19" s="9" t="n"/>
-      <c r="D19" s="6" t="n"/>
+      <c r="A19" s="14" t="n"/>
+      <c r="B19" s="18" t="n"/>
+      <c r="C19" s="18" t="n"/>
+      <c r="D19" s="18" t="n"/>
+      <c r="E19" s="18" t="n"/>
+      <c r="F19" s="18" t="n"/>
+      <c r="G19" s="18" t="n"/>
+      <c r="H19" s="18" t="n"/>
+      <c r="I19" s="18" t="n"/>
+      <c r="J19" s="18" t="n"/>
+      <c r="K19" s="18" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="4" t="n"/>
-      <c r="B20" s="8" t="n"/>
-      <c r="C20" s="8" t="n"/>
-      <c r="D20" s="4" t="n"/>
+      <c r="A20" s="16" t="n"/>
+      <c r="B20" s="19" t="n"/>
+      <c r="C20" s="19" t="n"/>
+      <c r="D20" s="19" t="n"/>
+      <c r="E20" s="19" t="n"/>
+      <c r="F20" s="19" t="n"/>
+      <c r="G20" s="19" t="n"/>
+      <c r="H20" s="19" t="n"/>
+      <c r="I20" s="19" t="n"/>
+      <c r="J20" s="19" t="n"/>
+      <c r="K20" s="19" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="6" t="n"/>
-      <c r="B21" s="9" t="n"/>
-      <c r="C21" s="9" t="n"/>
-      <c r="D21" s="6" t="n"/>
+      <c r="A21" s="14" t="n"/>
+      <c r="B21" s="18" t="n"/>
+      <c r="C21" s="18" t="n"/>
+      <c r="D21" s="18" t="n"/>
+      <c r="E21" s="18" t="n"/>
+      <c r="F21" s="18" t="n"/>
+      <c r="G21" s="18" t="n"/>
+      <c r="H21" s="18" t="n"/>
+      <c r="I21" s="18" t="n"/>
+      <c r="J21" s="18" t="n"/>
+      <c r="K21" s="18" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="4" t="n"/>
-      <c r="B22" s="8" t="n"/>
-      <c r="C22" s="8" t="n"/>
-      <c r="D22" s="4" t="n"/>
+      <c r="A22" s="16" t="n"/>
+      <c r="B22" s="19" t="n"/>
+      <c r="C22" s="19" t="n"/>
+      <c r="D22" s="19" t="n"/>
+      <c r="E22" s="19" t="n"/>
+      <c r="F22" s="19" t="n"/>
+      <c r="G22" s="19" t="n"/>
+      <c r="H22" s="19" t="n"/>
+      <c r="I22" s="19" t="n"/>
+      <c r="J22" s="19" t="n"/>
+      <c r="K22" s="19" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="6" t="n"/>
-      <c r="B23" s="9" t="n"/>
-      <c r="C23" s="9" t="n"/>
-      <c r="D23" s="6" t="n"/>
+      <c r="A23" s="14" t="n"/>
+      <c r="B23" s="18" t="n"/>
+      <c r="C23" s="18" t="n"/>
+      <c r="D23" s="18" t="n"/>
+      <c r="E23" s="18" t="n"/>
+      <c r="F23" s="18" t="n"/>
+      <c r="G23" s="18" t="n"/>
+      <c r="H23" s="18" t="n"/>
+      <c r="I23" s="18" t="n"/>
+      <c r="J23" s="18" t="n"/>
+      <c r="K23" s="18" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="16" t="n"/>
+      <c r="B24" s="19" t="n"/>
+      <c r="C24" s="19" t="n"/>
+      <c r="D24" s="19" t="n"/>
+      <c r="E24" s="19" t="n"/>
+      <c r="F24" s="19" t="n"/>
+      <c r="G24" s="19" t="n"/>
+      <c r="H24" s="19" t="n"/>
+      <c r="I24" s="19" t="n"/>
+      <c r="J24" s="19" t="n"/>
+      <c r="K24" s="19" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A2:D2"/>
+  <mergeCells count="7">
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="J3:K3"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="D3:E3"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="H3:I3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -809,288 +1228,288 @@
       </c>
     </row>
     <row r="2" ht="36" customHeight="1">
-      <c r="A2" s="10" t="inlineStr">
+      <c r="A2" s="20" t="inlineStr">
         <is>
           <t>Index</t>
         </is>
       </c>
-      <c r="B2" s="10" t="inlineStr">
+      <c r="B2" s="20" t="inlineStr">
         <is>
           <t>Formula</t>
         </is>
       </c>
-      <c r="C2" s="10" t="inlineStr">
+      <c r="C2" s="20" t="inlineStr">
         <is>
           <t>Desired Value</t>
         </is>
       </c>
-      <c r="D2" s="10" t="inlineStr">
+      <c r="D2" s="20" t="inlineStr">
         <is>
           <t>Interpretation</t>
         </is>
       </c>
-      <c r="E2" s="10" t="inlineStr">
+      <c r="E2" s="20" t="inlineStr">
         <is>
           <t>Reference</t>
         </is>
       </c>
-      <c r="F2" s="10" t="inlineStr">
+      <c r="F2" s="20" t="inlineStr">
         <is>
           <t>Sensitivity to High Yp</t>
         </is>
       </c>
     </row>
     <row r="3" ht="52" customHeight="1">
-      <c r="A3" s="11" t="inlineStr">
+      <c r="A3" s="21" t="inlineStr">
         <is>
           <t>TOL</t>
         </is>
       </c>
-      <c r="B3" s="12" t="inlineStr">
+      <c r="B3" s="22" t="inlineStr">
         <is>
           <t>Yp − Ys</t>
         </is>
       </c>
-      <c r="C3" s="11" t="inlineStr">
+      <c r="C3" s="21" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="D3" s="12" t="inlineStr">
+      <c r="D3" s="22" t="inlineStr">
         <is>
           <t>Absolute yield reduction under stress; lower = more stable.</t>
         </is>
       </c>
-      <c r="E3" s="11" t="inlineStr">
+      <c r="E3" s="21" t="inlineStr">
         <is>
           <t>Rosielle &amp; Hamblin (1981)</t>
         </is>
       </c>
-      <c r="F3" s="11" t="inlineStr">
+      <c r="F3" s="21" t="inlineStr">
         <is>
           <t>Insensitive</t>
         </is>
       </c>
     </row>
     <row r="4" ht="52" customHeight="1">
-      <c r="A4" s="13" t="inlineStr">
+      <c r="A4" s="23" t="inlineStr">
         <is>
           <t>MP</t>
         </is>
       </c>
-      <c r="B4" s="14" t="inlineStr">
+      <c r="B4" s="24" t="inlineStr">
         <is>
           <t>(Yp + Ys) / 2</t>
         </is>
       </c>
-      <c r="C4" s="13" t="inlineStr">
+      <c r="C4" s="23" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="D4" s="14" t="inlineStr">
+      <c r="D4" s="24" t="inlineStr">
         <is>
           <t>Average productivity across both environments.</t>
         </is>
       </c>
-      <c r="E4" s="13" t="inlineStr">
+      <c r="E4" s="23" t="inlineStr">
         <is>
           <t>Rosielle &amp; Hamblin (1981)</t>
         </is>
       </c>
-      <c r="F4" s="13" t="inlineStr">
+      <c r="F4" s="23" t="inlineStr">
         <is>
           <t>Sensitive</t>
         </is>
       </c>
     </row>
     <row r="5" ht="52" customHeight="1">
-      <c r="A5" s="11" t="inlineStr">
+      <c r="A5" s="21" t="inlineStr">
         <is>
           <t>GMP</t>
         </is>
       </c>
-      <c r="B5" s="12" t="inlineStr">
+      <c r="B5" s="22" t="inlineStr">
         <is>
           <t>√(Yp × Ys)</t>
         </is>
       </c>
-      <c r="C5" s="11" t="inlineStr">
+      <c r="C5" s="21" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="D5" s="12" t="inlineStr">
+      <c r="D5" s="22" t="inlineStr">
         <is>
           <t>Geometric mean; penalises large differences between Yp and Ys.</t>
         </is>
       </c>
-      <c r="E5" s="11" t="inlineStr">
+      <c r="E5" s="21" t="inlineStr">
         <is>
           <t>Fernandez (1992)</t>
         </is>
       </c>
-      <c r="F5" s="11" t="inlineStr">
+      <c r="F5" s="21" t="inlineStr">
         <is>
           <t>Moderately sensitive</t>
         </is>
       </c>
     </row>
     <row r="6" ht="52" customHeight="1">
-      <c r="A6" s="13" t="inlineStr">
+      <c r="A6" s="23" t="inlineStr">
         <is>
           <t>STI</t>
         </is>
       </c>
-      <c r="B6" s="14" t="inlineStr">
+      <c r="B6" s="24" t="inlineStr">
         <is>
           <t>(Yp × Ys) / mean(Yp)²</t>
         </is>
       </c>
-      <c r="C6" s="13" t="inlineStr">
+      <c r="C6" s="23" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="D6" s="14" t="inlineStr">
-        <is>
-          <t>Identifies genotypes with high yield under both conditions. STI &gt; 1 = above average in both environments.</t>
-        </is>
-      </c>
-      <c r="E6" s="13" t="inlineStr">
+      <c r="D6" s="24" t="inlineStr">
+        <is>
+          <t>Identifies genotypes with high yield under both conditions. STI &gt; 1 = above average in both.</t>
+        </is>
+      </c>
+      <c r="E6" s="23" t="inlineStr">
         <is>
           <t>Fernandez (1992)</t>
         </is>
       </c>
-      <c r="F6" s="13" t="inlineStr">
+      <c r="F6" s="23" t="inlineStr">
         <is>
           <t>Sensitive</t>
         </is>
       </c>
     </row>
     <row r="7" ht="52" customHeight="1">
-      <c r="A7" s="11" t="inlineStr">
+      <c r="A7" s="21" t="inlineStr">
         <is>
           <t>SSI</t>
         </is>
       </c>
-      <c r="B7" s="12" t="inlineStr">
+      <c r="B7" s="22" t="inlineStr">
         <is>
           <t>(1 − Ys/Yp) / (1 − mean(Ys)/mean(Yp))</t>
         </is>
       </c>
-      <c r="C7" s="11" t="inlineStr">
-        <is>
-          <t>Low  (&lt; 1)</t>
-        </is>
-      </c>
-      <c r="D7" s="12" t="inlineStr">
-        <is>
-          <t>Proportion of yield lost relative to population average. SSI &lt; 1 = tolerant; SSI &gt; 1 = sensitive.</t>
-        </is>
-      </c>
-      <c r="E7" s="11" t="inlineStr">
+      <c r="C7" s="21" t="inlineStr">
+        <is>
+          <t>Low (&lt; 1)</t>
+        </is>
+      </c>
+      <c r="D7" s="22" t="inlineStr">
+        <is>
+          <t>Proportion lost relative to population. SSI &lt; 1 = tolerant; SSI &gt; 1 = sensitive.</t>
+        </is>
+      </c>
+      <c r="E7" s="21" t="inlineStr">
         <is>
           <t>Fischer &amp; Maurer (1978)</t>
         </is>
       </c>
-      <c r="F7" s="11" t="inlineStr">
+      <c r="F7" s="21" t="inlineStr">
         <is>
           <t>Partially sensitive</t>
         </is>
       </c>
     </row>
     <row r="8" ht="52" customHeight="1">
-      <c r="A8" s="13" t="inlineStr">
+      <c r="A8" s="23" t="inlineStr">
         <is>
           <t>YSI</t>
         </is>
       </c>
-      <c r="B8" s="14" t="inlineStr">
+      <c r="B8" s="24" t="inlineStr">
         <is>
           <t>Ys / Yp</t>
         </is>
       </c>
-      <c r="C8" s="13" t="inlineStr">
-        <is>
-          <t>High  (→ 1)</t>
-        </is>
-      </c>
-      <c r="D8" s="14" t="inlineStr">
-        <is>
-          <t>Fraction of potential yield retained under stress. Closer to 1 = more tolerant.</t>
-        </is>
-      </c>
-      <c r="E8" s="13" t="inlineStr">
+      <c r="C8" s="23" t="inlineStr">
+        <is>
+          <t>High (→ 1)</t>
+        </is>
+      </c>
+      <c r="D8" s="24" t="inlineStr">
+        <is>
+          <t>Fraction of potential yield retained. Closer to 1 = more tolerant.</t>
+        </is>
+      </c>
+      <c r="E8" s="23" t="inlineStr">
         <is>
           <t>Bouslama &amp; Schapaugh (1984)</t>
         </is>
       </c>
-      <c r="F8" s="13" t="inlineStr">
+      <c r="F8" s="23" t="inlineStr">
         <is>
           <t>Insensitive</t>
         </is>
       </c>
     </row>
     <row r="9" ht="52" customHeight="1">
-      <c r="A9" s="11" t="inlineStr">
+      <c r="A9" s="21" t="inlineStr">
         <is>
           <t>HM</t>
         </is>
       </c>
-      <c r="B9" s="12" t="inlineStr">
+      <c r="B9" s="22" t="inlineStr">
         <is>
           <t>2·Yp·Ys / (Yp + Ys)</t>
         </is>
       </c>
-      <c r="C9" s="11" t="inlineStr">
+      <c r="C9" s="21" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="D9" s="12" t="inlineStr">
+      <c r="D9" s="22" t="inlineStr">
         <is>
           <t>Harmonic mean; more sensitive to the lower of the two values.</t>
         </is>
       </c>
-      <c r="E9" s="11" t="inlineStr">
+      <c r="E9" s="21" t="inlineStr">
         <is>
           <t>Kristin et al. (1993)</t>
         </is>
       </c>
-      <c r="F9" s="11" t="inlineStr">
+      <c r="F9" s="21" t="inlineStr">
         <is>
           <t>Moderately sensitive</t>
         </is>
       </c>
     </row>
     <row r="10" ht="52" customHeight="1">
-      <c r="A10" s="13" t="inlineStr">
+      <c r="A10" s="23" t="inlineStr">
         <is>
           <t>YI</t>
         </is>
       </c>
-      <c r="B10" s="14" t="inlineStr">
+      <c r="B10" s="24" t="inlineStr">
         <is>
           <t>Ys / mean(Ys)</t>
         </is>
       </c>
-      <c r="C10" s="13" t="inlineStr">
-        <is>
-          <t>High  (&gt; 1)</t>
-        </is>
-      </c>
-      <c r="D10" s="14" t="inlineStr">
-        <is>
-          <t>Relative stress yield compared to population mean. YI &gt; 1 = above-average stress performance.</t>
-        </is>
-      </c>
-      <c r="E10" s="13" t="inlineStr">
+      <c r="C10" s="23" t="inlineStr">
+        <is>
+          <t>High (&gt; 1)</t>
+        </is>
+      </c>
+      <c r="D10" s="24" t="inlineStr">
+        <is>
+          <t>Relative stress performance vs. population mean. YI &gt; 1 = above-average stress yield.</t>
+        </is>
+      </c>
+      <c r="E10" s="23" t="inlineStr">
         <is>
           <t>Fischer &amp; Maurer (1978)</t>
         </is>
       </c>
-      <c r="F10" s="13" t="inlineStr">
+      <c r="F10" s="23" t="inlineStr">
         <is>
           <t>Insensitive</t>
         </is>
@@ -1110,130 +1529,131 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="70" customWidth="1" min="2" max="2"/>
+    <col width="72" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="15" t="inlineStr">
+      <c r="A1" s="25" t="inlineStr">
         <is>
           <t>How to Use This Workbook with stress_tolerance_indices.R</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="52" customHeight="1">
-      <c r="A3" s="10" t="inlineStr">
+    <row r="3" ht="62" customHeight="1">
+      <c r="A3" s="20" t="inlineStr">
+        <is>
+          <t>Column naming
+rule</t>
+        </is>
+      </c>
+      <c r="B3" s="22" t="inlineStr">
+        <is>
+          <t>Each trait needs exactly TWO columns: TraitName_Yp (non-stress) and TraitName_Ys (stress).
+Example: GrainYield_Yp | GrainYield_Ys
+The R script detects all pairs automatically — add as many traits as you need.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="52" customHeight="1">
+      <c r="A4" s="20" t="inlineStr">
         <is>
           <t>Step 1</t>
         </is>
       </c>
-      <c r="B3" s="12" t="inlineStr">
-        <is>
-          <t>Open the 'Data' sheet and replace the sample genotype names and values with your own.  Keep the column headers exactly as they are (Genotype, Yp, Ys).</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="62" customHeight="1">
-      <c r="A4" s="10" t="inlineStr">
+      <c r="B4" s="24" t="inlineStr">
+        <is>
+          <t>Replace or add trait column pairs in the 'Data' sheet following the naming rule above.
+Keep 'Genotype' as the first column.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="52" customHeight="1">
+      <c r="A5" s="20" t="inlineStr">
         <is>
           <t>Step 2</t>
         </is>
       </c>
-      <c r="B4" s="14" t="inlineStr">
-        <is>
-          <t>Yp = yield or trait value measured in the NON-STRESS environment.
-Ys = yield or trait value measured under the STRESS environment
-(drought, heat, salinity, waterlogging, etc.).</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="52" customHeight="1">
-      <c r="A5" s="10" t="inlineStr">
+      <c r="B5" s="22" t="inlineStr">
+        <is>
+          <t>Fill in Yp and Ys values for every genotype × trait combination.
+Leave a cell blank only if data is truly missing (the script skips missing values).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="52" customHeight="1">
+      <c r="A6" s="20" t="inlineStr">
         <is>
           <t>Step 3</t>
         </is>
       </c>
-      <c r="B5" s="12" t="inlineStr">
+      <c r="B6" s="24" t="inlineStr">
         <is>
           <t>Save the file as  sample_data.xlsx  in the same folder as the R script.</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="52" customHeight="1">
-      <c r="A6" s="10" t="inlineStr">
+    <row r="7" ht="52" customHeight="1">
+      <c r="A7" s="20" t="inlineStr">
         <is>
           <t>Step 4</t>
         </is>
       </c>
-      <c r="B6" s="14" t="inlineStr">
-        <is>
-          <t>Open stress_tolerance_indices.R in RStudio (or any R IDE).</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="116" customHeight="1">
-      <c r="A7" s="10" t="inlineStr">
-        <is>
-          <t>Step 5</t>
-        </is>
-      </c>
-      <c r="B7" s="12" t="inlineStr">
-        <is>
-          <t>Run the script.  It will:
-  • Read your data from this Excel file
-  • Calculate all 8 stress tolerance indices
-  • Print a ranked table to the Console
-  • Save results to  stress_tolerance_results.csv
-  • Save 4 publication-quality plots as PNG files</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="52" customHeight="1">
-      <c r="A8" s="10" t="inlineStr">
-        <is>
-          <t>Tip</t>
-        </is>
-      </c>
-      <c r="B8" s="14" t="inlineStr">
-        <is>
-          <t>You can add as many genotype rows as you need in the Data sheet.
-The R script handles any number of rows automatically.</t>
+      <c r="B7" s="22" t="inlineStr">
+        <is>
+          <t>Open  stress_tolerance_indices.R  in RStudio and run it.
+The script will process ALL traits in one go automatically.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="80" customHeight="1">
+      <c r="A8" s="20" t="inlineStr">
+        <is>
+          <t>Outputs</t>
+        </is>
+      </c>
+      <c r="B8" s="24" t="inlineStr">
+        <is>
+          <t>• stress_tolerance_results.xlsx — one sheet per trait + a cross-trait summary sheet
+• stress_tolerance_results.csv  — long-format CSV with all results
+• PNG plots for each trait (bar chart, biplot, lollipop)
+• One combined heatmap comparing STI across all traits</t>
         </is>
       </c>
     </row>
     <row r="9" ht="52" customHeight="1">
-      <c r="A9" s="10" t="inlineStr">
-        <is>
-          <t>Units</t>
-        </is>
-      </c>
-      <c r="B9" s="12" t="inlineStr">
-        <is>
-          <t>Yield is typically in t ha⁻¹ or g plant⁻¹, but any consistent unit works.
-All indices are unit-independent ratios or differences.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="52" customHeight="1">
-      <c r="A10" s="10" t="inlineStr">
+      <c r="A9" s="20" t="inlineStr">
         <is>
           <t>Required
 R packages</t>
         </is>
       </c>
-      <c r="B10" s="14" t="inlineStr">
-        <is>
-          <t>readxl, ggplot2, reshape2, ggcorrplot, dplyr, ggrepel
-The script installs missing packages automatically on first run.</t>
+      <c r="B9" s="22" t="inlineStr">
+        <is>
+          <t>readxl, openxlsx, ggplot2, reshape2, ggcorrplot, dplyr, ggrepel
+All missing packages are installed automatically on first run.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="52" customHeight="1">
+      <c r="A10" s="20" t="inlineStr">
+        <is>
+          <t>Tip</t>
+        </is>
+      </c>
+      <c r="B10" s="24" t="inlineStr">
+        <is>
+          <t>You can rename the sample traits (GrainYield, PlantHeight, etc.) to match your experiment.
+Any number of genotypes and any number of traits are supported.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A1:B1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>